<commit_message>
fix Women points for IMWA teams
</commit_message>
<xml_diff>
--- a/owlcms/src/main/resources/templates/competitionBook/IMWA-A4.xlsx
+++ b/owlcms/src/main/resources/templates/competitionBook/IMWA-A4.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28526"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28730"/>
   <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\lamyj\git\owlcms4\owlcms\src\main\resources\templates\competitionBook\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1C7DC4FB-B2EB-48D6-A475-E31AC3978022}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1C486673-C5B8-4F12-9037-5570854EA507}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="17520" tabRatio="447" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="495" yWindow="2265" windowWidth="21600" windowHeight="11295" tabRatio="447" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="C" sheetId="35" r:id="rId1"/>
@@ -8328,7 +8328,7 @@
         <v>159</v>
       </c>
       <c r="K12" s="10" t="s">
-        <v>115</v>
+        <v>160</v>
       </c>
       <c r="L12" s="10" t="s">
         <v>58</v>

</xml_diff>

<commit_message>
fix default values if not best N
</commit_message>
<xml_diff>
--- a/owlcms/src/main/resources/templates/competitionBook/IMWA-A4.xlsx
+++ b/owlcms/src/main/resources/templates/competitionBook/IMWA-A4.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28730"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28827"/>
   <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\lamyj\git\owlcms4\owlcms\src\main\resources\templates\competitionBook\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1C486673-C5B8-4F12-9037-5570854EA507}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9B9FE4FB-98BE-4DB2-96F2-6DCC2C9DE40C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="495" yWindow="2265" windowWidth="21600" windowHeight="11295" tabRatio="447" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="3375" yWindow="2565" windowWidth="21600" windowHeight="12105" tabRatio="447" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="C" sheetId="35" r:id="rId1"/>
@@ -30,7 +30,7 @@
     <definedName name="_xlnm.Print_Titles" localSheetId="2">'W6'!$1:$2</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="4">WB!$1:$2</definedName>
   </definedNames>
-  <calcPr calcId="191029"/>
+  <calcPr calcId="191029" iterate="1"/>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
       <xcalcf:calcFeatures>
@@ -189,9 +189,6 @@
     <t>${t.get("Lot")}</t>
   </si>
   <si>
-    <t>${t.get("Results.MenPerTeam")}</t>
-  </si>
-  <si>
     <t>${t.get("Results.Teams")}</t>
   </si>
   <si>
@@ -210,9 +207,6 @@
     <t>${t.get("CompetitionBook.MT_RightHeader")} - ${t.get("CompetitionBook.MT_LeftHeader")}</t>
   </si>
   <si>
-    <t>${t.get("Results.WomenPerTeam")}</t>
-  </si>
-  <si>
     <t>${t.get("Gender.F")}</t>
   </si>
   <si>
@@ -366,12 +360,6 @@
     <t>${group.weighInShortDateTime != "" ? (t.get("WeighInTime")+': '+group.weighInShortDateTime) : ""}</t>
   </si>
   <si>
-    <t>${competition.menPerTeamElseDefault}</t>
-  </si>
-  <si>
-    <t>${competition.womenPerTeamElseDefault}</t>
-  </si>
-  <si>
     <t>&lt;jx:forEach items="${mTot}" groupBy="category.code"&gt;</t>
   </si>
   <si>
@@ -535,6 +523,18 @@
   </si>
   <si>
     <t>${l.category}</t>
+  </si>
+  <si>
+    <t>${competition.menBestNElseDefault}</t>
+  </si>
+  <si>
+    <t>${competition.womenBestNElseDefault}</t>
+  </si>
+  <si>
+    <t>${t.get("Results.MenBestN")}</t>
+  </si>
+  <si>
+    <t>${t.get("Results.WomenBestN")}</t>
   </si>
 </sst>
 </file>
@@ -2135,10 +2135,10 @@
   <sheetData>
     <row r="1" spans="1:19" ht="18" x14ac:dyDescent="0.25">
       <c r="A1" s="44" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
       <c r="B1" s="102" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="C1" s="102"/>
       <c r="D1" s="102"/>
@@ -2148,18 +2148,18 @@
       <c r="H1" s="44"/>
       <c r="I1" s="44"/>
       <c r="J1" s="44" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="K1" s="45" t="s">
-        <v>76</v>
+        <v>74</v>
       </c>
     </row>
     <row r="2" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A2" s="44" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="B2" s="103" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
       <c r="C2" s="103"/>
       <c r="D2" s="103"/>
@@ -2169,18 +2169,18 @@
       <c r="H2" s="44"/>
       <c r="I2" s="44"/>
       <c r="J2" s="44" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
       <c r="K2" s="45" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
     </row>
     <row r="3" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A3" s="44" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
       <c r="B3" s="103" t="s">
-        <v>112</v>
+        <v>108</v>
       </c>
       <c r="C3" s="103"/>
       <c r="D3" s="103"/>
@@ -2207,24 +2207,24 @@
     </row>
     <row r="7" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
     </row>
     <row r="8" spans="1:19" s="3" customFormat="1" ht="20.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="47" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="B8" s="48"/>
       <c r="C8" s="48" t="s">
-        <v>84</v>
+        <v>82</v>
       </c>
       <c r="D8" s="45" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
       <c r="G8" s="48"/>
       <c r="H8" s="48"/>
       <c r="I8" t="s">
-        <v>85</v>
+        <v>83</v>
       </c>
       <c r="J8" s="48"/>
       <c r="L8" s="49"/>
@@ -2249,42 +2249,42 @@
     </row>
     <row r="10" spans="1:19" s="45" customFormat="1" x14ac:dyDescent="0.2">
       <c r="C10" s="44" t="s">
+        <v>84</v>
+      </c>
+      <c r="D10" s="45" t="s">
+        <v>85</v>
+      </c>
+      <c r="H10" s="44" t="s">
         <v>86</v>
       </c>
-      <c r="D10" s="45" t="s">
+      <c r="I10" s="45" t="s">
         <v>87</v>
       </c>
-      <c r="H10" s="44" t="s">
+      <c r="L10" s="44" t="s">
+        <v>112</v>
+      </c>
+      <c r="M10" s="45" t="s">
         <v>88</v>
-      </c>
-      <c r="I10" s="45" t="s">
-        <v>89</v>
-      </c>
-      <c r="L10" s="44" t="s">
-        <v>116</v>
-      </c>
-      <c r="M10" s="45" t="s">
-        <v>90</v>
       </c>
     </row>
     <row r="11" spans="1:19" x14ac:dyDescent="0.2">
       <c r="C11" s="44" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="D11" s="45" t="s">
-        <v>92</v>
+        <v>90</v>
       </c>
       <c r="E11" s="1"/>
       <c r="H11" s="44" t="s">
-        <v>93</v>
+        <v>91</v>
       </c>
       <c r="I11" s="45" t="s">
-        <v>94</v>
+        <v>92</v>
       </c>
       <c r="J11" s="45"/>
       <c r="K11" s="1"/>
       <c r="M11" s="45" t="s">
-        <v>95</v>
+        <v>93</v>
       </c>
       <c r="N11" s="1"/>
       <c r="P11"/>
@@ -2294,22 +2294,22 @@
     </row>
     <row r="12" spans="1:19" x14ac:dyDescent="0.2">
       <c r="C12" s="44" t="s">
-        <v>96</v>
+        <v>94</v>
       </c>
       <c r="D12" s="45" t="s">
-        <v>97</v>
+        <v>95</v>
       </c>
       <c r="E12" s="1"/>
       <c r="H12" s="44" t="s">
-        <v>98</v>
+        <v>96</v>
       </c>
       <c r="I12" s="45" t="s">
-        <v>99</v>
+        <v>97</v>
       </c>
       <c r="J12" s="45"/>
       <c r="K12" s="1"/>
       <c r="M12" s="45" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="N12" s="1"/>
       <c r="O12" s="45"/>
@@ -2319,15 +2319,15 @@
     </row>
     <row r="13" spans="1:19" x14ac:dyDescent="0.2">
       <c r="C13" s="44" t="s">
-        <v>101</v>
+        <v>99</v>
       </c>
       <c r="D13" s="52" t="s">
-        <v>102</v>
+        <v>100</v>
       </c>
       <c r="J13" s="1"/>
       <c r="K13" s="1"/>
       <c r="M13" t="s">
-        <v>103</v>
+        <v>101</v>
       </c>
       <c r="N13"/>
       <c r="S13"/>
@@ -2340,7 +2340,7 @@
       <c r="K14" s="45"/>
       <c r="L14" s="45"/>
       <c r="M14" s="45" t="s">
-        <v>104</v>
+        <v>102</v>
       </c>
       <c r="N14" s="45"/>
       <c r="O14" s="45"/>
@@ -3831,10 +3831,10 @@
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
-        <v>113</v>
+        <v>109</v>
       </c>
       <c r="B1" t="s">
-        <v>114</v>
+        <v>110</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.2">
@@ -5501,33 +5501,33 @@
         <v>29</v>
       </c>
       <c r="E1" s="107" t="s">
+        <v>57</v>
+      </c>
+      <c r="F1" s="107" t="s">
+        <v>58</v>
+      </c>
+      <c r="G1" s="107" t="s">
         <v>59</v>
       </c>
-      <c r="F1" s="107" t="s">
+      <c r="H1" s="107" t="s">
         <v>60</v>
       </c>
-      <c r="G1" s="107" t="s">
+      <c r="I1" s="109" t="s">
         <v>61</v>
-      </c>
-      <c r="H1" s="107" t="s">
-        <v>62</v>
-      </c>
-      <c r="I1" s="109" t="s">
-        <v>63</v>
       </c>
       <c r="J1" s="110"/>
       <c r="K1" s="110"/>
       <c r="L1" s="110"/>
       <c r="M1" s="110"/>
       <c r="N1" s="109" t="s">
-        <v>64</v>
+        <v>62</v>
       </c>
       <c r="O1" s="110"/>
       <c r="P1" s="110"/>
       <c r="Q1" s="110"/>
       <c r="R1" s="110"/>
       <c r="S1" s="104" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="T1" s="105"/>
     </row>
@@ -5550,10 +5550,10 @@
         <v>3</v>
       </c>
       <c r="L2" s="32" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="M2" s="56" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="N2" s="16">
         <v>1</v>
@@ -5565,21 +5565,21 @@
         <v>3</v>
       </c>
       <c r="Q2" s="32" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="R2" s="56" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="S2" s="31" t="s">
+        <v>63</v>
+      </c>
+      <c r="T2" s="56" t="s">
         <v>65</v>
-      </c>
-      <c r="T2" s="56" t="s">
-        <v>67</v>
       </c>
     </row>
     <row r="3" spans="1:23" s="18" customFormat="1" ht="16.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A3" s="57" t="s">
-        <v>108</v>
+        <v>104</v>
       </c>
       <c r="B3" s="58"/>
       <c r="C3" s="58"/>
@@ -5607,7 +5607,7 @@
     </row>
     <row r="5" spans="1:23" ht="21.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A5" s="61" t="s">
-        <v>109</v>
+        <v>105</v>
       </c>
       <c r="B5" s="62"/>
       <c r="C5" s="63"/>
@@ -5634,7 +5634,7 @@
     </row>
     <row r="6" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
-        <v>110</v>
+        <v>106</v>
       </c>
       <c r="D6"/>
       <c r="E6"/>
@@ -5688,7 +5688,7 @@
         <v>36</v>
       </c>
       <c r="M7" s="55" t="s">
-        <v>155</v>
+        <v>151</v>
       </c>
       <c r="N7" s="25" t="s">
         <v>37</v>
@@ -5703,13 +5703,13 @@
         <v>40</v>
       </c>
       <c r="R7" s="55" t="s">
-        <v>156</v>
+        <v>152</v>
       </c>
       <c r="S7" s="23" t="s">
         <v>4</v>
       </c>
       <c r="T7" s="54" t="s">
-        <v>157</v>
+        <v>153</v>
       </c>
     </row>
     <row r="8" spans="1:23" x14ac:dyDescent="0.2">
@@ -6137,33 +6137,33 @@
         <v>29</v>
       </c>
       <c r="E1" s="107" t="s">
+        <v>57</v>
+      </c>
+      <c r="F1" s="107" t="s">
+        <v>58</v>
+      </c>
+      <c r="G1" s="107" t="s">
         <v>59</v>
       </c>
-      <c r="F1" s="107" t="s">
+      <c r="H1" s="107" t="s">
         <v>60</v>
       </c>
-      <c r="G1" s="107" t="s">
+      <c r="I1" s="109" t="s">
         <v>61</v>
-      </c>
-      <c r="H1" s="107" t="s">
-        <v>62</v>
-      </c>
-      <c r="I1" s="109" t="s">
-        <v>63</v>
       </c>
       <c r="J1" s="110"/>
       <c r="K1" s="110"/>
       <c r="L1" s="110"/>
       <c r="M1" s="110"/>
       <c r="N1" s="109" t="s">
-        <v>64</v>
+        <v>62</v>
       </c>
       <c r="O1" s="110"/>
       <c r="P1" s="110"/>
       <c r="Q1" s="110"/>
       <c r="R1" s="110"/>
       <c r="S1" s="104" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="T1" s="105"/>
     </row>
@@ -6186,10 +6186,10 @@
         <v>3</v>
       </c>
       <c r="L2" s="32" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="M2" s="56" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="N2" s="16">
         <v>1</v>
@@ -6201,21 +6201,21 @@
         <v>3</v>
       </c>
       <c r="Q2" s="32" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="R2" s="56" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="S2" s="31" t="s">
+        <v>63</v>
+      </c>
+      <c r="T2" s="56" t="s">
         <v>65</v>
-      </c>
-      <c r="T2" s="56" t="s">
-        <v>67</v>
       </c>
     </row>
     <row r="3" spans="1:23" s="18" customFormat="1" ht="16.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A3" s="57" t="s">
-        <v>111</v>
+        <v>107</v>
       </c>
       <c r="B3" s="58"/>
       <c r="C3" s="58"/>
@@ -6243,7 +6243,7 @@
     </row>
     <row r="5" spans="1:23" ht="21.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A5" s="61" t="s">
-        <v>109</v>
+        <v>105</v>
       </c>
       <c r="B5" s="62"/>
       <c r="C5" s="63"/>
@@ -6270,7 +6270,7 @@
     </row>
     <row r="6" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
-        <v>110</v>
+        <v>106</v>
       </c>
       <c r="D6"/>
       <c r="E6"/>
@@ -6322,7 +6322,7 @@
         <v>36</v>
       </c>
       <c r="M7" s="55" t="s">
-        <v>155</v>
+        <v>151</v>
       </c>
       <c r="N7" s="25" t="s">
         <v>37</v>
@@ -6337,13 +6337,13 @@
         <v>40</v>
       </c>
       <c r="R7" s="55" t="s">
-        <v>156</v>
+        <v>152</v>
       </c>
       <c r="S7" s="23" t="s">
         <v>4</v>
       </c>
       <c r="T7" s="54" t="s">
-        <v>157</v>
+        <v>153</v>
       </c>
     </row>
     <row r="8" spans="1:23" x14ac:dyDescent="0.2">
@@ -6769,34 +6769,34 @@
         <v>29</v>
       </c>
       <c r="E1" s="107" t="s">
+        <v>57</v>
+      </c>
+      <c r="F1" s="125" t="s">
+        <v>58</v>
+      </c>
+      <c r="G1" s="126" t="s">
         <v>59</v>
       </c>
-      <c r="F1" s="125" t="s">
+      <c r="H1" s="127" t="s">
         <v>60</v>
       </c>
-      <c r="G1" s="126" t="s">
+      <c r="I1" s="129" t="s">
         <v>61</v>
-      </c>
-      <c r="H1" s="127" t="s">
-        <v>62</v>
-      </c>
-      <c r="I1" s="129" t="s">
-        <v>63</v>
       </c>
       <c r="J1" s="129"/>
       <c r="K1" s="129"/>
       <c r="L1" s="129"/>
       <c r="M1" s="129" t="s">
-        <v>64</v>
+        <v>62</v>
       </c>
       <c r="N1" s="129"/>
       <c r="O1" s="129"/>
       <c r="P1" s="129"/>
       <c r="Q1" s="130" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="R1" s="119" t="s">
-        <v>149</v>
+        <v>145</v>
       </c>
       <c r="S1" s="119"/>
       <c r="U1"/>
@@ -6837,15 +6837,15 @@
       </c>
       <c r="Q2" s="131"/>
       <c r="R2" s="31" t="s">
-        <v>150</v>
+        <v>146</v>
       </c>
       <c r="S2" s="56" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
     </row>
     <row r="3" spans="1:22" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
-        <v>151</v>
+        <v>147</v>
       </c>
       <c r="D3"/>
       <c r="E3"/>
@@ -6877,7 +6877,7 @@
       </c>
       <c r="D4" s="17"/>
       <c r="E4" s="27" t="s">
-        <v>152</v>
+        <v>148</v>
       </c>
       <c r="F4" s="28" t="s">
         <v>2</v>
@@ -6916,10 +6916,10 @@
         <v>4</v>
       </c>
       <c r="R4" s="35" t="s">
-        <v>153</v>
+        <v>149</v>
       </c>
       <c r="S4" s="34" t="s">
-        <v>158</v>
+        <v>154</v>
       </c>
       <c r="V4" s="20" t="s">
         <v>41</v>
@@ -7315,34 +7315,34 @@
         <v>29</v>
       </c>
       <c r="E1" s="107" t="s">
+        <v>57</v>
+      </c>
+      <c r="F1" s="125" t="s">
+        <v>58</v>
+      </c>
+      <c r="G1" s="126" t="s">
         <v>59</v>
       </c>
-      <c r="F1" s="125" t="s">
+      <c r="H1" s="127" t="s">
         <v>60</v>
       </c>
-      <c r="G1" s="126" t="s">
+      <c r="I1" s="129" t="s">
         <v>61</v>
-      </c>
-      <c r="H1" s="127" t="s">
-        <v>62</v>
-      </c>
-      <c r="I1" s="129" t="s">
-        <v>63</v>
       </c>
       <c r="J1" s="129"/>
       <c r="K1" s="129"/>
       <c r="L1" s="129"/>
       <c r="M1" s="129" t="s">
-        <v>64</v>
+        <v>62</v>
       </c>
       <c r="N1" s="129"/>
       <c r="O1" s="129"/>
       <c r="P1" s="129"/>
       <c r="Q1" s="130" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="R1" s="119" t="s">
-        <v>149</v>
+        <v>145</v>
       </c>
       <c r="S1" s="119"/>
     </row>
@@ -7381,15 +7381,15 @@
       </c>
       <c r="Q2" s="131"/>
       <c r="R2" s="31" t="s">
-        <v>150</v>
+        <v>146</v>
       </c>
       <c r="S2" s="56" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
     </row>
     <row r="3" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
-        <v>154</v>
+        <v>150</v>
       </c>
       <c r="D3"/>
       <c r="E3"/>
@@ -7418,7 +7418,7 @@
       </c>
       <c r="D4" s="17"/>
       <c r="E4" s="27" t="s">
-        <v>152</v>
+        <v>148</v>
       </c>
       <c r="F4" s="28" t="s">
         <v>2</v>
@@ -7457,10 +7457,10 @@
         <v>4</v>
       </c>
       <c r="R4" s="35" t="s">
-        <v>153</v>
+        <v>149</v>
       </c>
       <c r="S4" s="34" t="s">
-        <v>158</v>
+        <v>154</v>
       </c>
     </row>
     <row r="5" spans="1:19" x14ac:dyDescent="0.2">
@@ -7819,7 +7819,7 @@
   <sheetData>
     <row r="1" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A1" s="14" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="B1" s="3"/>
       <c r="C1" s="3"/>
@@ -7830,28 +7830,28 @@
     </row>
     <row r="3" spans="1:19" s="6" customFormat="1" ht="39" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A3" s="43" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="B3" s="42" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="C3" s="42" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="D3" s="68" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="M3" s="43" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="N3" s="42" t="s">
-        <v>140</v>
+        <v>136</v>
       </c>
       <c r="O3" s="68" t="s">
-        <v>141</v>
+        <v>137</v>
       </c>
       <c r="P3" s="68" t="s">
-        <v>142</v>
+        <v>138</v>
       </c>
     </row>
     <row r="4" spans="1:19" x14ac:dyDescent="0.2">
@@ -7884,13 +7884,13 @@
         <v>13</v>
       </c>
       <c r="N5" s="40" t="s">
-        <v>143</v>
+        <v>139</v>
       </c>
       <c r="O5" s="40" t="s">
-        <v>144</v>
+        <v>140</v>
       </c>
       <c r="P5" s="100" t="s">
-        <v>145</v>
+        <v>141</v>
       </c>
     </row>
     <row r="6" spans="1:19" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
@@ -7913,7 +7913,7 @@
     </row>
     <row r="8" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A8" s="3" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="B8" s="3"/>
       <c r="C8" s="3"/>
@@ -7921,7 +7921,7 @@
     <row r="9" spans="1:19" ht="13.5" thickBot="1" x14ac:dyDescent="0.25"/>
     <row r="10" spans="1:19" ht="40.15" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A10" s="67" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="B10" s="39" t="s">
         <v>45</v>
@@ -7930,16 +7930,16 @@
         <v>44</v>
       </c>
       <c r="D10" s="39" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="E10" s="39" t="s">
-        <v>161</v>
+        <v>157</v>
       </c>
       <c r="F10" s="39" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="G10" s="7" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="H10" s="7" t="s">
         <v>8</v>
@@ -7948,25 +7948,25 @@
         <v>15</v>
       </c>
       <c r="J10" s="7" t="s">
+        <v>67</v>
+      </c>
+      <c r="K10" s="7" t="s">
+        <v>68</v>
+      </c>
+      <c r="L10" s="7" t="s">
         <v>69</v>
       </c>
-      <c r="K10" s="7" t="s">
+      <c r="M10" s="38" t="s">
         <v>70</v>
       </c>
-      <c r="L10" s="7" t="s">
-        <v>71</v>
-      </c>
-      <c r="M10" s="38" t="s">
-        <v>72</v>
-      </c>
       <c r="N10" s="38" t="s">
-        <v>140</v>
+        <v>136</v>
       </c>
       <c r="O10" s="38" t="s">
-        <v>141</v>
+        <v>137</v>
       </c>
       <c r="P10" s="68" t="s">
-        <v>142</v>
+        <v>138</v>
       </c>
     </row>
     <row r="11" spans="1:19" x14ac:dyDescent="0.2">
@@ -7995,7 +7995,7 @@
         <v>11</v>
       </c>
       <c r="E12" s="21" t="s">
-        <v>162</v>
+        <v>158</v>
       </c>
       <c r="F12" s="11" t="s">
         <v>10</v>
@@ -8010,25 +8010,25 @@
         <v>7</v>
       </c>
       <c r="J12" s="10" t="s">
-        <v>159</v>
+        <v>155</v>
       </c>
       <c r="K12" s="10" t="s">
-        <v>160</v>
+        <v>156</v>
       </c>
       <c r="L12" s="10" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="M12" s="66" t="s">
         <v>19</v>
       </c>
       <c r="N12" s="66" t="s">
-        <v>146</v>
+        <v>142</v>
       </c>
       <c r="O12" s="66" t="s">
-        <v>147</v>
+        <v>143</v>
       </c>
       <c r="P12" s="66" t="s">
-        <v>148</v>
+        <v>144</v>
       </c>
     </row>
     <row r="13" spans="1:19" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
@@ -8066,7 +8066,7 @@
     </row>
     <row r="15" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A15" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="C15" t="s">
         <v>23</v>
@@ -8074,7 +8074,7 @@
     </row>
     <row r="16" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A16" s="4" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="B16" s="5"/>
       <c r="C16" t="s">
@@ -8083,10 +8083,10 @@
     </row>
     <row r="17" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A17" t="s">
-        <v>47</v>
+        <v>161</v>
       </c>
       <c r="C17" t="s">
-        <v>106</v>
+        <v>159</v>
       </c>
     </row>
   </sheetData>
@@ -8134,7 +8134,7 @@
   <sheetData>
     <row r="1" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A1" s="14" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
       <c r="B1" s="3"/>
       <c r="C1" s="3"/>
@@ -8145,28 +8145,28 @@
     </row>
     <row r="3" spans="1:19" s="6" customFormat="1" ht="39" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A3" s="43" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="B3" s="42" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="C3" s="42" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="D3" s="68" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="M3" s="43" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="N3" s="42" t="s">
-        <v>140</v>
+        <v>136</v>
       </c>
       <c r="O3" s="68" t="s">
-        <v>141</v>
+        <v>137</v>
       </c>
       <c r="P3" s="68" t="s">
-        <v>142</v>
+        <v>138</v>
       </c>
     </row>
     <row r="4" spans="1:19" x14ac:dyDescent="0.2">
@@ -8199,13 +8199,13 @@
         <v>13</v>
       </c>
       <c r="N5" s="40" t="s">
-        <v>143</v>
+        <v>139</v>
       </c>
       <c r="O5" s="40" t="s">
-        <v>144</v>
+        <v>140</v>
       </c>
       <c r="P5" s="100" t="s">
-        <v>145</v>
+        <v>141</v>
       </c>
     </row>
     <row r="6" spans="1:19" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
@@ -8228,7 +8228,7 @@
     </row>
     <row r="8" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A8" s="3" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="B8" s="3"/>
       <c r="C8" s="3"/>
@@ -8236,7 +8236,7 @@
     <row r="9" spans="1:19" ht="13.5" thickBot="1" x14ac:dyDescent="0.25"/>
     <row r="10" spans="1:19" ht="40.15" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A10" s="67" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="B10" s="39" t="s">
         <v>45</v>
@@ -8245,16 +8245,16 @@
         <v>44</v>
       </c>
       <c r="D10" s="39" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="E10" s="39" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="F10" s="39" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="G10" s="7" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="H10" s="7" t="s">
         <v>8</v>
@@ -8263,25 +8263,25 @@
         <v>15</v>
       </c>
       <c r="J10" s="7" t="s">
+        <v>67</v>
+      </c>
+      <c r="K10" s="7" t="s">
+        <v>68</v>
+      </c>
+      <c r="L10" s="7" t="s">
         <v>69</v>
       </c>
-      <c r="K10" s="7" t="s">
+      <c r="M10" s="38" t="s">
         <v>70</v>
       </c>
-      <c r="L10" s="7" t="s">
-        <v>71</v>
-      </c>
-      <c r="M10" s="38" t="s">
-        <v>72</v>
-      </c>
       <c r="N10" s="38" t="s">
-        <v>140</v>
+        <v>136</v>
       </c>
       <c r="O10" s="38" t="s">
-        <v>141</v>
+        <v>137</v>
       </c>
       <c r="P10" s="68" t="s">
-        <v>142</v>
+        <v>138</v>
       </c>
     </row>
     <row r="11" spans="1:19" x14ac:dyDescent="0.2">
@@ -8325,25 +8325,25 @@
         <v>7</v>
       </c>
       <c r="J12" s="10" t="s">
-        <v>159</v>
+        <v>155</v>
       </c>
       <c r="K12" s="10" t="s">
-        <v>160</v>
+        <v>156</v>
       </c>
       <c r="L12" s="10" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="M12" s="66" t="s">
         <v>19</v>
       </c>
       <c r="N12" s="66" t="s">
-        <v>146</v>
+        <v>142</v>
       </c>
       <c r="O12" s="66" t="s">
-        <v>147</v>
+        <v>143</v>
       </c>
       <c r="P12" s="66" t="s">
-        <v>148</v>
+        <v>144</v>
       </c>
     </row>
     <row r="13" spans="1:19" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
@@ -8381,7 +8381,7 @@
     </row>
     <row r="15" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A15" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="C15" t="s">
         <v>25</v>
@@ -8389,7 +8389,7 @@
     </row>
     <row r="16" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A16" s="4" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="B16" s="5"/>
       <c r="C16" t="s">
@@ -8398,10 +8398,10 @@
     </row>
     <row r="18" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A18" t="s">
-        <v>54</v>
+        <v>162</v>
       </c>
       <c r="C18" t="s">
-        <v>107</v>
+        <v>160</v>
       </c>
     </row>
   </sheetData>
@@ -8449,7 +8449,7 @@
   <sheetData>
     <row r="1" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A1" s="14" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="B1" s="3"/>
       <c r="C1" s="3"/>
@@ -8460,31 +8460,31 @@
     </row>
     <row r="3" spans="1:19" s="6" customFormat="1" ht="39" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A3" s="43" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="B3" s="42" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="C3" s="42" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="D3" s="42" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="E3" s="68" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="M3" s="43" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="N3" s="42" t="s">
-        <v>140</v>
+        <v>136</v>
       </c>
       <c r="O3" s="68" t="s">
-        <v>141</v>
+        <v>137</v>
       </c>
       <c r="P3" s="68" t="s">
-        <v>142</v>
+        <v>138</v>
       </c>
     </row>
     <row r="4" spans="1:19" x14ac:dyDescent="0.2">
@@ -8520,13 +8520,13 @@
         <v>13</v>
       </c>
       <c r="N5" s="40" t="s">
-        <v>143</v>
+        <v>139</v>
       </c>
       <c r="O5" s="40" t="s">
-        <v>144</v>
+        <v>140</v>
       </c>
       <c r="P5" s="100" t="s">
-        <v>145</v>
+        <v>141</v>
       </c>
     </row>
     <row r="6" spans="1:19" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
@@ -8550,7 +8550,7 @@
     </row>
     <row r="8" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A8" s="3" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="B8" s="3"/>
       <c r="C8" s="3"/>
@@ -8558,7 +8558,7 @@
     <row r="9" spans="1:19" ht="13.5" thickBot="1" x14ac:dyDescent="0.25"/>
     <row r="10" spans="1:19" ht="41.45" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A10" s="67" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="B10" s="39" t="s">
         <v>45</v>
@@ -8567,16 +8567,16 @@
         <v>44</v>
       </c>
       <c r="D10" s="39" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="E10" s="39" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="F10" s="39" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="G10" s="7" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="H10" s="7" t="s">
         <v>8</v>
@@ -8585,25 +8585,25 @@
         <v>15</v>
       </c>
       <c r="J10" s="7" t="s">
+        <v>67</v>
+      </c>
+      <c r="K10" s="7" t="s">
+        <v>68</v>
+      </c>
+      <c r="L10" s="7" t="s">
         <v>69</v>
       </c>
-      <c r="K10" s="7" t="s">
+      <c r="M10" s="38" t="s">
         <v>70</v>
       </c>
-      <c r="L10" s="7" t="s">
-        <v>71</v>
-      </c>
-      <c r="M10" s="38" t="s">
-        <v>72</v>
-      </c>
       <c r="N10" s="38" t="s">
-        <v>140</v>
+        <v>136</v>
       </c>
       <c r="O10" s="38" t="s">
-        <v>141</v>
+        <v>137</v>
       </c>
       <c r="P10" s="68" t="s">
-        <v>142</v>
+        <v>138</v>
       </c>
     </row>
     <row r="11" spans="1:19" x14ac:dyDescent="0.2">
@@ -8647,25 +8647,25 @@
         <v>7</v>
       </c>
       <c r="J12" s="10" t="s">
-        <v>159</v>
+        <v>155</v>
       </c>
       <c r="K12" s="10" t="s">
-        <v>115</v>
+        <v>111</v>
       </c>
       <c r="L12" s="10" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="M12" s="66" t="s">
         <v>19</v>
       </c>
       <c r="N12" s="66" t="s">
-        <v>146</v>
+        <v>142</v>
       </c>
       <c r="O12" s="66" t="s">
-        <v>147</v>
+        <v>143</v>
       </c>
       <c r="P12" s="66" t="s">
-        <v>148</v>
+        <v>144</v>
       </c>
     </row>
     <row r="13" spans="1:19" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
@@ -8703,7 +8703,7 @@
     </row>
     <row r="15" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A15" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="C15" t="s">
         <v>43</v>
@@ -8711,7 +8711,7 @@
     </row>
     <row r="16" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A16" s="4" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="B16" s="5"/>
       <c r="C16" t="s">
@@ -8720,18 +8720,18 @@
     </row>
     <row r="17" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A17" t="s">
-        <v>47</v>
+        <v>161</v>
       </c>
       <c r="C17" t="s">
-        <v>106</v>
+        <v>159</v>
       </c>
     </row>
     <row r="18" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A18" t="s">
-        <v>54</v>
+        <v>162</v>
       </c>
       <c r="C18" t="s">
-        <v>107</v>
+        <v>160</v>
       </c>
     </row>
   </sheetData>
@@ -8781,13 +8781,13 @@
   <sheetData>
     <row r="1" spans="1:24" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
-        <v>117</v>
+        <v>113</v>
       </c>
       <c r="J1" s="1"/>
     </row>
     <row r="2" spans="1:24" s="69" customFormat="1" ht="15" x14ac:dyDescent="0.25">
       <c r="A2" s="69" t="s">
-        <v>118</v>
+        <v>114</v>
       </c>
       <c r="J2" s="70"/>
     </row>
@@ -8817,54 +8817,54 @@
     </row>
     <row r="4" spans="1:24" s="82" customFormat="1" ht="12" x14ac:dyDescent="0.2">
       <c r="A4" s="73" t="s">
-        <v>119</v>
+        <v>115</v>
       </c>
       <c r="B4" s="74"/>
       <c r="C4" s="75"/>
       <c r="D4" s="76" t="s">
-        <v>120</v>
+        <v>116</v>
       </c>
       <c r="E4" s="77" t="s">
-        <v>121</v>
+        <v>117</v>
       </c>
       <c r="F4" s="76" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="G4" s="78" t="s">
-        <v>122</v>
+        <v>118</v>
       </c>
       <c r="H4" s="79"/>
       <c r="I4" s="76" t="s">
-        <v>123</v>
+        <v>119</v>
       </c>
       <c r="J4" s="73" t="s">
-        <v>124</v>
+        <v>120</v>
       </c>
       <c r="K4" s="80"/>
       <c r="L4" s="74"/>
       <c r="M4" s="75"/>
       <c r="N4" s="73" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="O4" s="74"/>
       <c r="P4" s="81"/>
       <c r="Q4" s="73" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="R4" s="74"/>
       <c r="S4" s="73" t="s">
-        <v>125</v>
+        <v>121</v>
       </c>
       <c r="T4" s="80"/>
       <c r="U4" s="73" t="s">
-        <v>126</v>
+        <v>122</v>
       </c>
       <c r="V4" s="81"/>
       <c r="X4" s="75"/>
     </row>
     <row r="5" spans="1:24" s="87" customFormat="1" ht="16.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A5" s="83" t="s">
-        <v>127</v>
+        <v>123</v>
       </c>
       <c r="B5" s="84"/>
       <c r="C5" s="84"/>
@@ -8880,47 +8880,47 @@
     </row>
     <row r="6" spans="1:24" s="96" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A6" s="88" t="s">
-        <v>128</v>
+        <v>124</v>
       </c>
       <c r="B6" s="89"/>
       <c r="C6" s="90"/>
       <c r="D6" s="91" t="s">
-        <v>129</v>
+        <v>125</v>
       </c>
       <c r="E6" s="92" t="s">
-        <v>130</v>
+        <v>126</v>
       </c>
       <c r="F6" s="88" t="s">
-        <v>131</v>
+        <v>127</v>
       </c>
       <c r="G6" s="92" t="s">
-        <v>139</v>
+        <v>135</v>
       </c>
       <c r="H6" s="90"/>
       <c r="I6" s="94" t="s">
-        <v>132</v>
+        <v>128</v>
       </c>
       <c r="J6" s="92" t="s">
-        <v>138</v>
+        <v>134</v>
       </c>
       <c r="K6" s="89"/>
       <c r="L6" s="89"/>
       <c r="M6" s="90"/>
       <c r="N6" s="92" t="s">
-        <v>133</v>
+        <v>129</v>
       </c>
       <c r="O6" s="89"/>
       <c r="P6" s="90"/>
       <c r="Q6" s="88" t="s">
-        <v>134</v>
+        <v>130</v>
       </c>
       <c r="R6" s="89"/>
       <c r="S6" s="93" t="s">
-        <v>135</v>
+        <v>131</v>
       </c>
       <c r="T6" s="89"/>
       <c r="U6" s="95" t="s">
-        <v>136</v>
+        <v>132</v>
       </c>
       <c r="V6" s="90"/>
       <c r="X6" s="90"/>
@@ -8947,7 +8947,7 @@
     </row>
     <row r="8" spans="1:24" s="96" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A8" s="96" t="s">
-        <v>137</v>
+        <v>133</v>
       </c>
       <c r="B8" s="84"/>
       <c r="C8" s="84"/>

</xml_diff>